<commit_message>
feat: checkpoint Luoyang world and final asset integration
</commit_message>
<xml_diff>
--- a/Docs/KNOWLEDGE_BASE/REGISTRY/DESIGN_DECISION_REGISTRY.xlsx
+++ b/Docs/KNOWLEDGE_BASE/REGISTRY/DESIGN_DECISION_REGISTRY.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="说明" sheetId="1" r:id="R30d5c047573d4f1e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数据" sheetId="2" r:id="R590f2e1f23b24f8a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="说明" sheetId="1" r:id="Rb5eedbc7fd1340bf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数据" sheetId="2" r:id="Rc5d7032184334a57"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -576,8 +576,7 @@
         <x:v>记录数</x:v>
       </x:c>
       <x:c r="B2" s="7" t="n">
-        <x:f>COUNTA(A4:A5)</x:f>
-        <x:v>2</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="30" customHeight="1">
@@ -629,6 +628,40 @@
       </x:c>
       <x:c r="E5" t="str">
         <x:v>追加V72智能决策、Arena、模型和后续缺口记录；既有行保持不变。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" t="str">
+        <x:v>DESIGN_DECISION_REGISTRY.xlsx</x:v>
+      </x:c>
+      <x:c r="B6" t="str">
+        <x:v>LUOYANG-184-T4-LIVING-WORLD-COMPLETION-MASTER-V1</x:v>
+      </x:c>
+      <x:c r="C6" t="n">
+        <x:v>104</x:v>
+      </x:c>
+      <x:c r="D6" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E6" t="str">
+        <x:v>追加洛阳T4 Phase 0—19正式状态、完成证据与Deferred边界；既有行保持不变。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" t="str">
+        <x:v>DESIGN_DECISION_REGISTRY.xlsx</x:v>
+      </x:c>
+      <x:c r="B7" t="str">
+        <x:v>HAN-WORLD-STYLE-D-STRATEGIC-LANDSCAPE-VISUAL-REFINEMENT-AND-ZHONGHUA-SOURCE-RECOVERY-V2</x:v>
+      </x:c>
+      <x:c r="C7" t="str">
+        <x:v>140</x:v>
+      </x:c>
+      <x:c r="D7" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E7" t="str">
+        <x:v>登记Style D V2表现分辨率与正式Cell分辨率分离的冻结决策；不改世界事实。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -637,7 +670,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7cf390a6239b4a26"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R76dca74aee5d477a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -682,8 +715,7 @@
         <x:v>记录数</x:v>
       </x:c>
       <x:c r="B2" s="7" t="n">
-        <x:f>COUNTA(A4:A107)</x:f>
-        <x:v>104</x:v>
+        <x:v>141</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="30" customHeight="1">
@@ -4441,13 +4473,1211 @@
         <x:v>V72</x:v>
       </x:c>
     </x:row>
+    <x:row r="108">
+      <x:c r="A108" t="str">
+        <x:v>DEC-LUOYANG-T4-001</x:v>
+      </x:c>
+      <x:c r="B108" t="str">
+        <x:v>LuoyangLivingWorld</x:v>
+      </x:c>
+      <x:c r="C108" t="str">
+        <x:v>洛阳T4先完整后全国扩张</x:v>
+      </x:c>
+      <x:c r="D108" t="str">
+        <x:v>保留40万人、80899家户、2084开局设施；真实Cell、资源、资金、Order/Shipment、AI与历史事件共用同一世界事实</x:v>
+      </x:c>
+      <x:c r="E108" t="str">
+        <x:v>FROZEN</x:v>
+      </x:c>
+      <x:c r="F108" t="str">
+        <x:v>2026-08-12</x:v>
+      </x:c>
+      <x:c r="G108" t="str">
+        <x:v>Docs/TASK_LUOYANG_184_T4_LIVING_WORLD_COMPLETION_MASTER_V1.md</x:v>
+      </x:c>
+      <x:c r="H108"/>
+      <x:c r="I108" t="str">
+        <x:v>Docs/GAME_SYSTEMS_MASTER_AND_STATUS.md</x:v>
+      </x:c>
+      <x:c r="J108" t="str">
+        <x:v>Population|Property|Economy|AI|Government|Military|History</x:v>
+      </x:c>
+      <x:c r="K108" t="str">
+        <x:v>先把洛阳做活、做完整，再恢复全国Runtime扩张</x:v>
+      </x:c>
+      <x:c r="L108"/>
+      <x:c r="M108" t="str">
+        <x:v>T4 Living World V1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="109">
+      <x:c r="A109" t="str">
+        <x:v>decision.map-presentation.01.v1</x:v>
+      </x:c>
+      <x:c r="B109" t="str">
+        <x:v>MapPresentation</x:v>
+      </x:c>
+      <x:c r="C109" t="str">
+        <x:v>Map presentation decision 1</x:v>
+      </x:c>
+      <x:c r="D109" t="str">
+        <x:v>Simulation Cell remains authoritative; visual anchors do not create SubCells.</x:v>
+      </x:c>
+      <x:c r="E109" t="str">
+        <x:v>ACCEPTED</x:v>
+      </x:c>
+      <x:c r="F109" t="str">
+        <x:v>2026-08-12</x:v>
+      </x:c>
+      <x:c r="G109" t="str">
+        <x:v>Docs/TASK_LUOYANG_PLAYABLE_VERTICAL_SLICE_MAP_PRESENTATION_AND_CONSTRUCTION_ASSET_LIBRARY_V1.md</x:v>
+      </x:c>
+      <x:c r="H109" t="str"/>
+      <x:c r="I109" t="str"/>
+      <x:c r="J109" t="str">
+        <x:v>Map|Construction|Facility|Population|Persistence</x:v>
+      </x:c>
+      <x:c r="K109" t="str">
+        <x:v>Preserve one world while adding reusable player-visible presentation.</x:v>
+      </x:c>
+      <x:c r="L109" t="str"/>
+      <x:c r="M109" t="str"/>
+    </x:row>
+    <x:row r="110">
+      <x:c r="A110" t="str">
+        <x:v>decision.map-presentation.02.v1</x:v>
+      </x:c>
+      <x:c r="B110" t="str">
+        <x:v>MapPresentation</x:v>
+      </x:c>
+      <x:c r="C110" t="str">
+        <x:v>Map presentation decision 2</x:v>
+      </x:c>
+      <x:c r="D110" t="str">
+        <x:v>Simulation Facility may use multiple visual meshes and modules.</x:v>
+      </x:c>
+      <x:c r="E110" t="str">
+        <x:v>ACCEPTED</x:v>
+      </x:c>
+      <x:c r="F110" t="str">
+        <x:v>2026-08-12</x:v>
+      </x:c>
+      <x:c r="G110" t="str">
+        <x:v>Docs/TASK_LUOYANG_PLAYABLE_VERTICAL_SLICE_MAP_PRESENTATION_AND_CONSTRUCTION_ASSET_LIBRARY_V1.md</x:v>
+      </x:c>
+      <x:c r="H110" t="str"/>
+      <x:c r="I110" t="str"/>
+      <x:c r="J110" t="str">
+        <x:v>Map|Construction|Facility|Population|Persistence</x:v>
+      </x:c>
+      <x:c r="K110" t="str">
+        <x:v>Preserve one world while adding reusable player-visible presentation.</x:v>
+      </x:c>
+      <x:c r="L110" t="str"/>
+      <x:c r="M110" t="str"/>
+    </x:row>
+    <x:row r="111">
+      <x:c r="A111" t="str">
+        <x:v>decision.map-presentation.03.v1</x:v>
+      </x:c>
+      <x:c r="B111" t="str">
+        <x:v>MapPresentation</x:v>
+      </x:c>
+      <x:c r="C111" t="str">
+        <x:v>Map presentation decision 3</x:v>
+      </x:c>
+      <x:c r="D111" t="str">
+        <x:v>Historical initialization, AI construction and player construction reuse the same formal construction asset system.</x:v>
+      </x:c>
+      <x:c r="E111" t="str">
+        <x:v>ACCEPTED</x:v>
+      </x:c>
+      <x:c r="F111" t="str">
+        <x:v>2026-08-12</x:v>
+      </x:c>
+      <x:c r="G111" t="str">
+        <x:v>Docs/TASK_LUOYANG_PLAYABLE_VERTICAL_SLICE_MAP_PRESENTATION_AND_CONSTRUCTION_ASSET_LIBRARY_V1.md</x:v>
+      </x:c>
+      <x:c r="H111" t="str"/>
+      <x:c r="I111" t="str"/>
+      <x:c r="J111" t="str">
+        <x:v>Map|Construction|Facility|Population|Persistence</x:v>
+      </x:c>
+      <x:c r="K111" t="str">
+        <x:v>Preserve one world while adding reusable player-visible presentation.</x:v>
+      </x:c>
+      <x:c r="L111" t="str"/>
+      <x:c r="M111" t="str"/>
+    </x:row>
+    <x:row r="112">
+      <x:c r="A112" t="str">
+        <x:v>decision.map-presentation.04.v1</x:v>
+      </x:c>
+      <x:c r="B112" t="str">
+        <x:v>MapPresentation</x:v>
+      </x:c>
+      <x:c r="C112" t="str">
+        <x:v>Map presentation decision 4</x:v>
+      </x:c>
+      <x:c r="D112" t="str">
+        <x:v>Historical unique compositions may be HistoricalInitOnly while reusing common modular kits.</x:v>
+      </x:c>
+      <x:c r="E112" t="str">
+        <x:v>ACCEPTED</x:v>
+      </x:c>
+      <x:c r="F112" t="str">
+        <x:v>2026-08-12</x:v>
+      </x:c>
+      <x:c r="G112" t="str">
+        <x:v>Docs/TASK_LUOYANG_PLAYABLE_VERTICAL_SLICE_MAP_PRESENTATION_AND_CONSTRUCTION_ASSET_LIBRARY_V1.md</x:v>
+      </x:c>
+      <x:c r="H112" t="str"/>
+      <x:c r="I112" t="str"/>
+      <x:c r="J112" t="str">
+        <x:v>Map|Construction|Facility|Population|Persistence</x:v>
+      </x:c>
+      <x:c r="K112" t="str">
+        <x:v>Preserve one world while adding reusable player-visible presentation.</x:v>
+      </x:c>
+      <x:c r="L112" t="str"/>
+      <x:c r="M112" t="str"/>
+    </x:row>
+    <x:row r="113">
+      <x:c r="A113" t="str">
+        <x:v>decision.map-presentation.05.v1</x:v>
+      </x:c>
+      <x:c r="B113" t="str">
+        <x:v>MapPresentation</x:v>
+      </x:c>
+      <x:c r="C113" t="str">
+        <x:v>Map presentation decision 5</x:v>
+      </x:c>
+      <x:c r="D113" t="str">
+        <x:v>Core scene buildings must bind to Runtime Facility IDs.</x:v>
+      </x:c>
+      <x:c r="E113" t="str">
+        <x:v>ACCEPTED</x:v>
+      </x:c>
+      <x:c r="F113" t="str">
+        <x:v>2026-08-12</x:v>
+      </x:c>
+      <x:c r="G113" t="str">
+        <x:v>Docs/TASK_LUOYANG_PLAYABLE_VERTICAL_SLICE_MAP_PRESENTATION_AND_CONSTRUCTION_ASSET_LIBRARY_V1.md</x:v>
+      </x:c>
+      <x:c r="H113" t="str"/>
+      <x:c r="I113" t="str"/>
+      <x:c r="J113" t="str">
+        <x:v>Map|Construction|Facility|Population|Persistence</x:v>
+      </x:c>
+      <x:c r="K113" t="str">
+        <x:v>Preserve one world while adding reusable player-visible presentation.</x:v>
+      </x:c>
+      <x:c r="L113" t="str"/>
+      <x:c r="M113" t="str"/>
+    </x:row>
+    <x:row r="114">
+      <x:c r="A114" t="str">
+        <x:v>decision.map-presentation.06.v1</x:v>
+      </x:c>
+      <x:c r="B114" t="str">
+        <x:v>MapPresentation</x:v>
+      </x:c>
+      <x:c r="C114" t="str">
+        <x:v>Map presentation decision 6</x:v>
+      </x:c>
+      <x:c r="D114" t="str">
+        <x:v>Decorative props do not require Facility IDs.</x:v>
+      </x:c>
+      <x:c r="E114" t="str">
+        <x:v>ACCEPTED</x:v>
+      </x:c>
+      <x:c r="F114" t="str">
+        <x:v>2026-08-12</x:v>
+      </x:c>
+      <x:c r="G114" t="str">
+        <x:v>Docs/TASK_LUOYANG_PLAYABLE_VERTICAL_SLICE_MAP_PRESENTATION_AND_CONSTRUCTION_ASSET_LIBRARY_V1.md</x:v>
+      </x:c>
+      <x:c r="H114" t="str"/>
+      <x:c r="I114" t="str"/>
+      <x:c r="J114" t="str">
+        <x:v>Map|Construction|Facility|Population|Persistence</x:v>
+      </x:c>
+      <x:c r="K114" t="str">
+        <x:v>Preserve one world while adding reusable player-visible presentation.</x:v>
+      </x:c>
+      <x:c r="L114" t="str"/>
+      <x:c r="M114" t="str"/>
+    </x:row>
+    <x:row r="115">
+      <x:c r="A115" t="str">
+        <x:v>decision.map-presentation.07.v1</x:v>
+      </x:c>
+      <x:c r="B115" t="str">
+        <x:v>MapPresentation</x:v>
+      </x:c>
+      <x:c r="C115" t="str">
+        <x:v>Map presentation decision 7</x:v>
+      </x:c>
+      <x:c r="D115" t="str">
+        <x:v>Normal gameplay hides Cell grid; Build and analysis modes may reveal it.</x:v>
+      </x:c>
+      <x:c r="E115" t="str">
+        <x:v>ACCEPTED</x:v>
+      </x:c>
+      <x:c r="F115" t="str">
+        <x:v>2026-08-12</x:v>
+      </x:c>
+      <x:c r="G115" t="str">
+        <x:v>Docs/TASK_LUOYANG_PLAYABLE_VERTICAL_SLICE_MAP_PRESENTATION_AND_CONSTRUCTION_ASSET_LIBRARY_V1.md</x:v>
+      </x:c>
+      <x:c r="H115" t="str"/>
+      <x:c r="I115" t="str"/>
+      <x:c r="J115" t="str">
+        <x:v>Map|Construction|Facility|Population|Persistence</x:v>
+      </x:c>
+      <x:c r="K115" t="str">
+        <x:v>Preserve one world while adding reusable player-visible presentation.</x:v>
+      </x:c>
+      <x:c r="L115" t="str"/>
+      <x:c r="M115" t="str"/>
+    </x:row>
+    <x:row r="116">
+      <x:c r="A116" t="str">
+        <x:v>decision.map-presentation.08.v1</x:v>
+      </x:c>
+      <x:c r="B116" t="str">
+        <x:v>MapPresentation</x:v>
+      </x:c>
+      <x:c r="C116" t="str">
+        <x:v>Map presentation decision 8</x:v>
+      </x:c>
+      <x:c r="D116" t="str">
+        <x:v>Map zoom changes presentation LOD, not world truth.</x:v>
+      </x:c>
+      <x:c r="E116" t="str">
+        <x:v>ACCEPTED</x:v>
+      </x:c>
+      <x:c r="F116" t="str">
+        <x:v>2026-08-12</x:v>
+      </x:c>
+      <x:c r="G116" t="str">
+        <x:v>Docs/TASK_LUOYANG_PLAYABLE_VERTICAL_SLICE_MAP_PRESENTATION_AND_CONSTRUCTION_ASSET_LIBRARY_V1.md</x:v>
+      </x:c>
+      <x:c r="H116" t="str"/>
+      <x:c r="I116" t="str"/>
+      <x:c r="J116" t="str">
+        <x:v>Map|Construction|Facility|Population|Persistence</x:v>
+      </x:c>
+      <x:c r="K116" t="str">
+        <x:v>Preserve one world while adding reusable player-visible presentation.</x:v>
+      </x:c>
+      <x:c r="L116" t="str"/>
+      <x:c r="M116" t="str"/>
+    </x:row>
+    <x:row r="117">
+      <x:c r="A117" t="str">
+        <x:v>decision.map-presentation.09.v1</x:v>
+      </x:c>
+      <x:c r="B117" t="str">
+        <x:v>MapPresentation</x:v>
+      </x:c>
+      <x:c r="C117" t="str">
+        <x:v>Map presentation decision 9</x:v>
+      </x:c>
+      <x:c r="D117" t="str">
+        <x:v>Crop visual state derives from runtime crop state.</x:v>
+      </x:c>
+      <x:c r="E117" t="str">
+        <x:v>ACCEPTED</x:v>
+      </x:c>
+      <x:c r="F117" t="str">
+        <x:v>2026-08-12</x:v>
+      </x:c>
+      <x:c r="G117" t="str">
+        <x:v>Docs/TASK_LUOYANG_PLAYABLE_VERTICAL_SLICE_MAP_PRESENTATION_AND_CONSTRUCTION_ASSET_LIBRARY_V1.md</x:v>
+      </x:c>
+      <x:c r="H117" t="str"/>
+      <x:c r="I117" t="str"/>
+      <x:c r="J117" t="str">
+        <x:v>Map|Construction|Facility|Population|Persistence</x:v>
+      </x:c>
+      <x:c r="K117" t="str">
+        <x:v>Preserve one world while adding reusable player-visible presentation.</x:v>
+      </x:c>
+      <x:c r="L117" t="str"/>
+      <x:c r="M117" t="str"/>
+    </x:row>
+    <x:row r="118">
+      <x:c r="A118" t="str">
+        <x:v>decision.map-presentation.10.v1</x:v>
+      </x:c>
+      <x:c r="B118" t="str">
+        <x:v>MapPresentation</x:v>
+      </x:c>
+      <x:c r="C118" t="str">
+        <x:v>Map presentation decision 10</x:v>
+      </x:c>
+      <x:c r="D118" t="str">
+        <x:v>Shipment representation derives from runtime Shipment.</x:v>
+      </x:c>
+      <x:c r="E118" t="str">
+        <x:v>ACCEPTED</x:v>
+      </x:c>
+      <x:c r="F118" t="str">
+        <x:v>2026-08-12</x:v>
+      </x:c>
+      <x:c r="G118" t="str">
+        <x:v>Docs/TASK_LUOYANG_PLAYABLE_VERTICAL_SLICE_MAP_PRESENTATION_AND_CONSTRUCTION_ASSET_LIBRARY_V1.md</x:v>
+      </x:c>
+      <x:c r="H118" t="str"/>
+      <x:c r="I118" t="str"/>
+      <x:c r="J118" t="str">
+        <x:v>Map|Construction|Facility|Population|Persistence</x:v>
+      </x:c>
+      <x:c r="K118" t="str">
+        <x:v>Preserve one world while adding reusable player-visible presentation.</x:v>
+      </x:c>
+      <x:c r="L118" t="str"/>
+      <x:c r="M118" t="str"/>
+    </x:row>
+    <x:row r="119">
+      <x:c r="A119" t="str">
+        <x:v>decision.map-presentation.11.v1</x:v>
+      </x:c>
+      <x:c r="B119" t="str">
+        <x:v>MapPresentation</x:v>
+      </x:c>
+      <x:c r="C119" t="str">
+        <x:v>Map presentation decision 11</x:v>
+      </x:c>
+      <x:c r="D119" t="str">
+        <x:v>Person visual actors are temporary representations of PermanentPerson records.</x:v>
+      </x:c>
+      <x:c r="E119" t="str">
+        <x:v>ACCEPTED</x:v>
+      </x:c>
+      <x:c r="F119" t="str">
+        <x:v>2026-08-12</x:v>
+      </x:c>
+      <x:c r="G119" t="str">
+        <x:v>Docs/TASK_LUOYANG_PLAYABLE_VERTICAL_SLICE_MAP_PRESENTATION_AND_CONSTRUCTION_ASSET_LIBRARY_V1.md</x:v>
+      </x:c>
+      <x:c r="H119" t="str"/>
+      <x:c r="I119" t="str"/>
+      <x:c r="J119" t="str">
+        <x:v>Map|Construction|Facility|Population|Persistence</x:v>
+      </x:c>
+      <x:c r="K119" t="str">
+        <x:v>Preserve one world while adding reusable player-visible presentation.</x:v>
+      </x:c>
+      <x:c r="L119" t="str"/>
+      <x:c r="M119" t="str"/>
+    </x:row>
+    <x:row r="120">
+      <x:c r="A120" t="str">
+        <x:v>decision.map-presentation.12.v1</x:v>
+      </x:c>
+      <x:c r="B120" t="str">
+        <x:v>MapPresentation</x:v>
+      </x:c>
+      <x:c r="C120" t="str">
+        <x:v>Map presentation decision 12</x:v>
+      </x:c>
+      <x:c r="D120" t="str">
+        <x:v>Regional architectural styles change VisualProfile, not FacilityDefinition.</x:v>
+      </x:c>
+      <x:c r="E120" t="str">
+        <x:v>ACCEPTED</x:v>
+      </x:c>
+      <x:c r="F120" t="str">
+        <x:v>2026-08-12</x:v>
+      </x:c>
+      <x:c r="G120" t="str">
+        <x:v>Docs/TASK_LUOYANG_PLAYABLE_VERTICAL_SLICE_MAP_PRESENTATION_AND_CONSTRUCTION_ASSET_LIBRARY_V1.md</x:v>
+      </x:c>
+      <x:c r="H120" t="str"/>
+      <x:c r="I120" t="str"/>
+      <x:c r="J120" t="str">
+        <x:v>Map|Construction|Facility|Population|Persistence</x:v>
+      </x:c>
+      <x:c r="K120" t="str">
+        <x:v>Preserve one world while adding reusable player-visible presentation.</x:v>
+      </x:c>
+      <x:c r="L120" t="str"/>
+      <x:c r="M120" t="str"/>
+    </x:row>
+    <x:row r="121">
+      <x:c r="A121" t="str">
+        <x:v>decision.global-spatial.01.v1</x:v>
+      </x:c>
+      <x:c r="B121" t="str">
+        <x:v>GlobalSpatialFoundation</x:v>
+      </x:c>
+      <x:c r="C121" t="str">
+        <x:v>Global spatial foundation decision 1</x:v>
+      </x:c>
+      <x:c r="D121" t="str">
+        <x:v>Global CRS is the only authoritative geographic coordinate system.</x:v>
+      </x:c>
+      <x:c r="E121" t="str">
+        <x:v>ACCEPTED</x:v>
+      </x:c>
+      <x:c r="F121" t="str">
+        <x:v>2026-08-15</x:v>
+      </x:c>
+      <x:c r="G121" t="str">
+        <x:v>Docs/HISTORICAL_WORLD_REFERENCE/WORLD_GLOBAL_ORIGIN_CELL_GRID_AND_SPATIAL_CONTINUITY_V1/GLOBAL_SPATIAL_FOUNDATION_CONTRACT_V1.md</x:v>
+      </x:c>
+      <x:c r="H121" t="str"/>
+      <x:c r="I121" t="str"/>
+      <x:c r="J121" t="str">
+        <x:v>Map|GIS|Cell|Chunk|Terrain|Road|River|Place|Persistence|Presentation</x:v>
+      </x:c>
+      <x:c r="K121" t="str">
+        <x:v>Preserve one continuous national world and stable spatial identities.</x:v>
+      </x:c>
+      <x:c r="L121" t="str"/>
+      <x:c r="M121" t="str"/>
+    </x:row>
+    <x:row r="122">
+      <x:c r="A122" t="str">
+        <x:v>decision.global-spatial.02.v1</x:v>
+      </x:c>
+      <x:c r="B122" t="str">
+        <x:v>GlobalSpatialFoundation</x:v>
+      </x:c>
+      <x:c r="C122" t="str">
+        <x:v>Global spatial foundation decision 2</x:v>
+      </x:c>
+      <x:c r="D122" t="str">
+        <x:v>Global Origin and Global Cell Grid are one unified spatial contract.</x:v>
+      </x:c>
+      <x:c r="E122" t="str">
+        <x:v>ACCEPTED</x:v>
+      </x:c>
+      <x:c r="F122" t="str">
+        <x:v>2026-08-15</x:v>
+      </x:c>
+      <x:c r="G122" t="str">
+        <x:v>Docs/HISTORICAL_WORLD_REFERENCE/WORLD_GLOBAL_ORIGIN_CELL_GRID_AND_SPATIAL_CONTINUITY_V1/GLOBAL_SPATIAL_FOUNDATION_CONTRACT_V1.md</x:v>
+      </x:c>
+      <x:c r="H122" t="str"/>
+      <x:c r="I122" t="str"/>
+      <x:c r="J122" t="str">
+        <x:v>Map|GIS|Cell|Chunk|Terrain|Road|River|Place|Persistence|Presentation</x:v>
+      </x:c>
+      <x:c r="K122" t="str">
+        <x:v>Preserve one continuous national world and stable spatial identities.</x:v>
+      </x:c>
+      <x:c r="L122" t="str"/>
+      <x:c r="M122" t="str"/>
+    </x:row>
+    <x:row r="123">
+      <x:c r="A123" t="str">
+        <x:v>decision.global-spatial.03.v1</x:v>
+      </x:c>
+      <x:c r="B123" t="str">
+        <x:v>GlobalSpatialFoundation</x:v>
+      </x:c>
+      <x:c r="C123" t="str">
+        <x:v>Global spatial foundation decision 3</x:v>
+      </x:c>
+      <x:c r="D123" t="str">
+        <x:v>All regions reuse the same Global Cell Grid.</x:v>
+      </x:c>
+      <x:c r="E123" t="str">
+        <x:v>ACCEPTED</x:v>
+      </x:c>
+      <x:c r="F123" t="str">
+        <x:v>2026-08-15</x:v>
+      </x:c>
+      <x:c r="G123" t="str">
+        <x:v>Docs/HISTORICAL_WORLD_REFERENCE/WORLD_GLOBAL_ORIGIN_CELL_GRID_AND_SPATIAL_CONTINUITY_V1/GLOBAL_SPATIAL_FOUNDATION_CONTRACT_V1.md</x:v>
+      </x:c>
+      <x:c r="H123" t="str"/>
+      <x:c r="I123" t="str"/>
+      <x:c r="J123" t="str">
+        <x:v>Map|GIS|Cell|Chunk|Terrain|Road|River|Place|Persistence|Presentation</x:v>
+      </x:c>
+      <x:c r="K123" t="str">
+        <x:v>Preserve one continuous national world and stable spatial identities.</x:v>
+      </x:c>
+      <x:c r="L123" t="str"/>
+      <x:c r="M123" t="str"/>
+    </x:row>
+    <x:row r="124">
+      <x:c r="A124" t="str">
+        <x:v>decision.global-spatial.04.v1</x:v>
+      </x:c>
+      <x:c r="B124" t="str">
+        <x:v>GlobalSpatialFoundation</x:v>
+      </x:c>
+      <x:c r="C124" t="str">
+        <x:v>Global spatial foundation decision 4</x:v>
+      </x:c>
+      <x:c r="D124" t="str">
+        <x:v>Region Local Coordinates are reversible presentation/editor coordinates, not new world coordinates.</x:v>
+      </x:c>
+      <x:c r="E124" t="str">
+        <x:v>ACCEPTED</x:v>
+      </x:c>
+      <x:c r="F124" t="str">
+        <x:v>2026-08-15</x:v>
+      </x:c>
+      <x:c r="G124" t="str">
+        <x:v>Docs/HISTORICAL_WORLD_REFERENCE/WORLD_GLOBAL_ORIGIN_CELL_GRID_AND_SPATIAL_CONTINUITY_V1/GLOBAL_SPATIAL_FOUNDATION_CONTRACT_V1.md</x:v>
+      </x:c>
+      <x:c r="H124" t="str"/>
+      <x:c r="I124" t="str"/>
+      <x:c r="J124" t="str">
+        <x:v>Map|GIS|Cell|Chunk|Terrain|Road|River|Place|Persistence|Presentation</x:v>
+      </x:c>
+      <x:c r="K124" t="str">
+        <x:v>Preserve one continuous national world and stable spatial identities.</x:v>
+      </x:c>
+      <x:c r="L124" t="str"/>
+      <x:c r="M124" t="str"/>
+    </x:row>
+    <x:row r="125">
+      <x:c r="A125" t="str">
+        <x:v>decision.global-spatial.05.v1</x:v>
+      </x:c>
+      <x:c r="B125" t="str">
+        <x:v>GlobalSpatialFoundation</x:v>
+      </x:c>
+      <x:c r="C125" t="str">
+        <x:v>Global spatial foundation decision 5</x:v>
+      </x:c>
+      <x:c r="D125" t="str">
+        <x:v>Global Chunk Grid is derived from Global Cell Grid and is never re-cut by Region.</x:v>
+      </x:c>
+      <x:c r="E125" t="str">
+        <x:v>ACCEPTED</x:v>
+      </x:c>
+      <x:c r="F125" t="str">
+        <x:v>2026-08-15</x:v>
+      </x:c>
+      <x:c r="G125" t="str">
+        <x:v>Docs/HISTORICAL_WORLD_REFERENCE/WORLD_GLOBAL_ORIGIN_CELL_GRID_AND_SPATIAL_CONTINUITY_V1/GLOBAL_SPATIAL_FOUNDATION_CONTRACT_V1.md</x:v>
+      </x:c>
+      <x:c r="H125" t="str"/>
+      <x:c r="I125" t="str"/>
+      <x:c r="J125" t="str">
+        <x:v>Map|GIS|Cell|Chunk|Terrain|Road|River|Place|Persistence|Presentation</x:v>
+      </x:c>
+      <x:c r="K125" t="str">
+        <x:v>Preserve one continuous national world and stable spatial identities.</x:v>
+      </x:c>
+      <x:c r="L125" t="str"/>
+      <x:c r="M125" t="str"/>
+    </x:row>
+    <x:row r="126">
+      <x:c r="A126" t="str">
+        <x:v>decision.global-spatial.06.v1</x:v>
+      </x:c>
+      <x:c r="B126" t="str">
+        <x:v>GlobalSpatialFoundation</x:v>
+      </x:c>
+      <x:c r="C126" t="str">
+        <x:v>Global spatial foundation decision 6</x:v>
+      </x:c>
+      <x:c r="D126" t="str">
+        <x:v>DEM sampling is globally aligned before regional high-detail production.</x:v>
+      </x:c>
+      <x:c r="E126" t="str">
+        <x:v>ACCEPTED</x:v>
+      </x:c>
+      <x:c r="F126" t="str">
+        <x:v>2026-08-15</x:v>
+      </x:c>
+      <x:c r="G126" t="str">
+        <x:v>Docs/HISTORICAL_WORLD_REFERENCE/WORLD_GLOBAL_ORIGIN_CELL_GRID_AND_SPATIAL_CONTINUITY_V1/GLOBAL_SPATIAL_FOUNDATION_CONTRACT_V1.md</x:v>
+      </x:c>
+      <x:c r="H126" t="str"/>
+      <x:c r="I126" t="str"/>
+      <x:c r="J126" t="str">
+        <x:v>Map|GIS|Cell|Chunk|Terrain|Road|River|Place|Persistence|Presentation</x:v>
+      </x:c>
+      <x:c r="K126" t="str">
+        <x:v>Preserve one continuous national world and stable spatial identities.</x:v>
+      </x:c>
+      <x:c r="L126" t="str"/>
+      <x:c r="M126" t="str"/>
+    </x:row>
+    <x:row r="127">
+      <x:c r="A127" t="str">
+        <x:v>decision.global-spatial.07.v1</x:v>
+      </x:c>
+      <x:c r="B127" t="str">
+        <x:v>GlobalSpatialFoundation</x:v>
+      </x:c>
+      <x:c r="C127" t="str">
+        <x:v>Global spatial foundation decision 7</x:v>
+      </x:c>
+      <x:c r="D127" t="str">
+        <x:v>Visual Local Anchors do not create Facility SubCells.</x:v>
+      </x:c>
+      <x:c r="E127" t="str">
+        <x:v>ACCEPTED</x:v>
+      </x:c>
+      <x:c r="F127" t="str">
+        <x:v>2026-08-15</x:v>
+      </x:c>
+      <x:c r="G127" t="str">
+        <x:v>Docs/HISTORICAL_WORLD_REFERENCE/WORLD_GLOBAL_ORIGIN_CELL_GRID_AND_SPATIAL_CONTINUITY_V1/GLOBAL_SPATIAL_FOUNDATION_CONTRACT_V1.md</x:v>
+      </x:c>
+      <x:c r="H127" t="str"/>
+      <x:c r="I127" t="str"/>
+      <x:c r="J127" t="str">
+        <x:v>Map|GIS|Cell|Chunk|Terrain|Road|River|Place|Persistence|Presentation</x:v>
+      </x:c>
+      <x:c r="K127" t="str">
+        <x:v>Preserve one continuous national world and stable spatial identities.</x:v>
+      </x:c>
+      <x:c r="L127" t="str"/>
+      <x:c r="M127" t="str"/>
+    </x:row>
+    <x:row r="128">
+      <x:c r="A128" t="str">
+        <x:v>decision.global-spatial.08.v1</x:v>
+      </x:c>
+      <x:c r="B128" t="str">
+        <x:v>GlobalSpatialFoundation</x:v>
+      </x:c>
+      <x:c r="C128" t="str">
+        <x:v>Global spatial foundation decision 8</x:v>
+      </x:c>
+      <x:c r="D128" t="str">
+        <x:v>Floating Origin changes Unity presentation coordinates only.</x:v>
+      </x:c>
+      <x:c r="E128" t="str">
+        <x:v>ACCEPTED</x:v>
+      </x:c>
+      <x:c r="F128" t="str">
+        <x:v>2026-08-15</x:v>
+      </x:c>
+      <x:c r="G128" t="str">
+        <x:v>Docs/HISTORICAL_WORLD_REFERENCE/WORLD_GLOBAL_ORIGIN_CELL_GRID_AND_SPATIAL_CONTINUITY_V1/GLOBAL_SPATIAL_FOUNDATION_CONTRACT_V1.md</x:v>
+      </x:c>
+      <x:c r="H128" t="str"/>
+      <x:c r="I128" t="str"/>
+      <x:c r="J128" t="str">
+        <x:v>Map|GIS|Cell|Chunk|Terrain|Road|River|Place|Persistence|Presentation</x:v>
+      </x:c>
+      <x:c r="K128" t="str">
+        <x:v>Preserve one continuous national world and stable spatial identities.</x:v>
+      </x:c>
+      <x:c r="L128" t="str"/>
+      <x:c r="M128" t="str"/>
+    </x:row>
+    <x:row r="129">
+      <x:c r="A129" t="str">
+        <x:v>decision.global-spatial.09.v1</x:v>
+      </x:c>
+      <x:c r="B129" t="str">
+        <x:v>GlobalSpatialFoundation</x:v>
+      </x:c>
+      <x:c r="C129" t="str">
+        <x:v>Global spatial foundation decision 9</x:v>
+      </x:c>
+      <x:c r="D129" t="str">
+        <x:v>Administrative boundaries do not define Cell geometry.</x:v>
+      </x:c>
+      <x:c r="E129" t="str">
+        <x:v>ACCEPTED</x:v>
+      </x:c>
+      <x:c r="F129" t="str">
+        <x:v>2026-08-15</x:v>
+      </x:c>
+      <x:c r="G129" t="str">
+        <x:v>Docs/HISTORICAL_WORLD_REFERENCE/WORLD_GLOBAL_ORIGIN_CELL_GRID_AND_SPATIAL_CONTINUITY_V1/GLOBAL_SPATIAL_FOUNDATION_CONTRACT_V1.md</x:v>
+      </x:c>
+      <x:c r="H129" t="str"/>
+      <x:c r="I129" t="str"/>
+      <x:c r="J129" t="str">
+        <x:v>Map|GIS|Cell|Chunk|Terrain|Road|River|Place|Persistence|Presentation</x:v>
+      </x:c>
+      <x:c r="K129" t="str">
+        <x:v>Preserve one continuous national world and stable spatial identities.</x:v>
+      </x:c>
+      <x:c r="L129" t="str"/>
+      <x:c r="M129" t="str"/>
+    </x:row>
+    <x:row r="130">
+      <x:c r="A130" t="str">
+        <x:v>decision.global-spatial.10.v1</x:v>
+      </x:c>
+      <x:c r="B130" t="str">
+        <x:v>GlobalSpatialFoundation</x:v>
+      </x:c>
+      <x:c r="C130" t="str">
+        <x:v>Global spatial foundation decision 10</x:v>
+      </x:c>
+      <x:c r="D130" t="str">
+        <x:v>Map production is national-space-first and region-detail-second.</x:v>
+      </x:c>
+      <x:c r="E130" t="str">
+        <x:v>ACCEPTED</x:v>
+      </x:c>
+      <x:c r="F130" t="str">
+        <x:v>2026-08-15</x:v>
+      </x:c>
+      <x:c r="G130" t="str">
+        <x:v>Docs/HISTORICAL_WORLD_REFERENCE/WORLD_GLOBAL_ORIGIN_CELL_GRID_AND_SPATIAL_CONTINUITY_V1/GLOBAL_SPATIAL_FOUNDATION_CONTRACT_V1.md</x:v>
+      </x:c>
+      <x:c r="H130" t="str"/>
+      <x:c r="I130" t="str"/>
+      <x:c r="J130" t="str">
+        <x:v>Map|GIS|Cell|Chunk|Terrain|Road|River|Place|Persistence|Presentation</x:v>
+      </x:c>
+      <x:c r="K130" t="str">
+        <x:v>Preserve one continuous national world and stable spatial identities.</x:v>
+      </x:c>
+      <x:c r="L130" t="str"/>
+      <x:c r="M130" t="str"/>
+    </x:row>
+    <x:row r="131">
+      <x:c r="A131" t="str">
+        <x:v>decision.global-spatial.11.v1</x:v>
+      </x:c>
+      <x:c r="B131" t="str">
+        <x:v>GlobalSpatialFoundation</x:v>
+      </x:c>
+      <x:c r="C131" t="str">
+        <x:v>Global spatial foundation decision 11</x:v>
+      </x:c>
+      <x:c r="D131" t="str">
+        <x:v>Canonical Global Chunk is 16x16 Cells; legacy 64x64 blocks are compression storage only.</x:v>
+      </x:c>
+      <x:c r="E131" t="str">
+        <x:v>ACCEPTED</x:v>
+      </x:c>
+      <x:c r="F131" t="str">
+        <x:v>2026-08-15</x:v>
+      </x:c>
+      <x:c r="G131" t="str">
+        <x:v>Docs/HISTORICAL_WORLD_REFERENCE/WORLD_GLOBAL_ORIGIN_CELL_GRID_AND_SPATIAL_CONTINUITY_V1/GLOBAL_SPATIAL_FOUNDATION_CONTRACT_V1.md</x:v>
+      </x:c>
+      <x:c r="H131" t="str"/>
+      <x:c r="I131" t="str"/>
+      <x:c r="J131" t="str">
+        <x:v>Map|GIS|Cell|Chunk|Terrain|Road|River|Place|Persistence|Presentation</x:v>
+      </x:c>
+      <x:c r="K131" t="str">
+        <x:v>Preserve one continuous national world and stable spatial identities.</x:v>
+      </x:c>
+      <x:c r="L131" t="str"/>
+      <x:c r="M131" t="str"/>
+    </x:row>
+    <x:row r="132">
+      <x:c r="A132" t="str">
+        <x:v>decision.global-spatial.12.v1</x:v>
+      </x:c>
+      <x:c r="B132" t="str">
+        <x:v>GlobalSpatialFoundation</x:v>
+      </x:c>
+      <x:c r="C132" t="str">
+        <x:v>Global spatial foundation decision 12</x:v>
+      </x:c>
+      <x:c r="D132" t="str">
+        <x:v>Stable Cell IDs outrank cosmetic origin, row or chunk renumbering.</x:v>
+      </x:c>
+      <x:c r="E132" t="str">
+        <x:v>ACCEPTED</x:v>
+      </x:c>
+      <x:c r="F132" t="str">
+        <x:v>2026-08-15</x:v>
+      </x:c>
+      <x:c r="G132" t="str">
+        <x:v>Docs/HISTORICAL_WORLD_REFERENCE/WORLD_GLOBAL_ORIGIN_CELL_GRID_AND_SPATIAL_CONTINUITY_V1/GLOBAL_SPATIAL_FOUNDATION_CONTRACT_V1.md</x:v>
+      </x:c>
+      <x:c r="H132" t="str"/>
+      <x:c r="I132" t="str"/>
+      <x:c r="J132" t="str">
+        <x:v>Map|GIS|Cell|Chunk|Terrain|Road|River|Place|Persistence|Presentation</x:v>
+      </x:c>
+      <x:c r="K132" t="str">
+        <x:v>Preserve one continuous national world and stable spatial identities.</x:v>
+      </x:c>
+      <x:c r="L132" t="str"/>
+      <x:c r="M132" t="str"/>
+    </x:row>
+    <x:row r="133">
+      <x:c r="A133" t="str">
+        <x:v>decision.region-cell-boundary.01.v1</x:v>
+      </x:c>
+      <x:c r="B133" t="str">
+        <x:v>GlobalSpatialFoundation</x:v>
+      </x:c>
+      <x:c r="C133" t="str">
+        <x:v>Region and technical-block semantic decision 1</x:v>
+      </x:c>
+      <x:c r="D133" t="str">
+        <x:v>Global Cell Grid is the only authoritative spatial partition of the world.</x:v>
+      </x:c>
+      <x:c r="E133" t="str">
+        <x:v>ACCEPTED</x:v>
+      </x:c>
+      <x:c r="F133" t="str">
+        <x:v>2026-08-15</x:v>
+      </x:c>
+      <x:c r="G133" t="str">
+        <x:v>Docs/HISTORICAL_WORLD_REFERENCE/WORLD_GLOBAL_ORIGIN_CELL_GRID_AND_SPATIAL_CONTINUITY_V1/GLOBAL_SPATIAL_FOUNDATION_CONTRACT_V1.md</x:v>
+      </x:c>
+      <x:c r="H133" t="str"/>
+      <x:c r="I133" t="str"/>
+      <x:c r="J133" t="str">
+        <x:v>Map|GIS|Cell|Region|Simulation|Terrain|Streaming|Storage|Persistence|Presentation</x:v>
+      </x:c>
+      <x:c r="K133" t="str">
+        <x:v>Keep Global Cell as the final world-space fact while allowing benchmark-driven technical partition sizes.</x:v>
+      </x:c>
+      <x:c r="L133" t="str"/>
+      <x:c r="M133" t="str"/>
+    </x:row>
+    <x:row r="134">
+      <x:c r="A134" t="str">
+        <x:v>decision.region-cell-boundary.02.v1</x:v>
+      </x:c>
+      <x:c r="B134" t="str">
+        <x:v>GlobalSpatialFoundation</x:v>
+      </x:c>
+      <x:c r="C134" t="str">
+        <x:v>Region and technical-block semantic decision 2</x:v>
+      </x:c>
+      <x:c r="D134" t="str">
+        <x:v>Region is defined by membership of complete Global Cells.</x:v>
+      </x:c>
+      <x:c r="E134" t="str">
+        <x:v>ACCEPTED</x:v>
+      </x:c>
+      <x:c r="F134" t="str">
+        <x:v>2026-08-15</x:v>
+      </x:c>
+      <x:c r="G134" t="str">
+        <x:v>Docs/HISTORICAL_WORLD_REFERENCE/WORLD_GLOBAL_ORIGIN_CELL_GRID_AND_SPATIAL_CONTINUITY_V1/GLOBAL_SPATIAL_FOUNDATION_CONTRACT_V1.md</x:v>
+      </x:c>
+      <x:c r="H134" t="str"/>
+      <x:c r="I134" t="str"/>
+      <x:c r="J134" t="str">
+        <x:v>Map|GIS|Cell|Region|Simulation|Terrain|Streaming|Storage|Persistence|Presentation</x:v>
+      </x:c>
+      <x:c r="K134" t="str">
+        <x:v>Keep Global Cell as the final world-space fact while allowing benchmark-driven technical partition sizes.</x:v>
+      </x:c>
+      <x:c r="L134" t="str"/>
+      <x:c r="M134" t="str"/>
+    </x:row>
+    <x:row r="135">
+      <x:c r="A135" t="str">
+        <x:v>decision.region-cell-boundary.03.v1</x:v>
+      </x:c>
+      <x:c r="B135" t="str">
+        <x:v>GlobalSpatialFoundation</x:v>
+      </x:c>
+      <x:c r="C135" t="str">
+        <x:v>Region and technical-block semantic decision 3</x:v>
+      </x:c>
+      <x:c r="D135" t="str">
+        <x:v>Region boundary is derived from member Cell outer edges.</x:v>
+      </x:c>
+      <x:c r="E135" t="str">
+        <x:v>ACCEPTED</x:v>
+      </x:c>
+      <x:c r="F135" t="str">
+        <x:v>2026-08-15</x:v>
+      </x:c>
+      <x:c r="G135" t="str">
+        <x:v>Docs/HISTORICAL_WORLD_REFERENCE/WORLD_GLOBAL_ORIGIN_CELL_GRID_AND_SPATIAL_CONTINUITY_V1/GLOBAL_SPATIAL_FOUNDATION_CONTRACT_V1.md</x:v>
+      </x:c>
+      <x:c r="H135" t="str"/>
+      <x:c r="I135" t="str"/>
+      <x:c r="J135" t="str">
+        <x:v>Map|GIS|Cell|Region|Simulation|Terrain|Streaming|Storage|Persistence|Presentation</x:v>
+      </x:c>
+      <x:c r="K135" t="str">
+        <x:v>Keep Global Cell as the final world-space fact while allowing benchmark-driven technical partition sizes.</x:v>
+      </x:c>
+      <x:c r="L135" t="str"/>
+      <x:c r="M135" t="str"/>
+    </x:row>
+    <x:row r="136">
+      <x:c r="A136" t="str">
+        <x:v>decision.region-cell-boundary.04.v1</x:v>
+      </x:c>
+      <x:c r="B136" t="str">
+        <x:v>GlobalSpatialFoundation</x:v>
+      </x:c>
+      <x:c r="C136" t="str">
+        <x:v>Region and technical-block semantic decision 4</x:v>
+      </x:c>
+      <x:c r="D136" t="str">
+        <x:v>Region boundaries never split Global Cells.</x:v>
+      </x:c>
+      <x:c r="E136" t="str">
+        <x:v>ACCEPTED</x:v>
+      </x:c>
+      <x:c r="F136" t="str">
+        <x:v>2026-08-15</x:v>
+      </x:c>
+      <x:c r="G136" t="str">
+        <x:v>Docs/HISTORICAL_WORLD_REFERENCE/WORLD_GLOBAL_ORIGIN_CELL_GRID_AND_SPATIAL_CONTINUITY_V1/GLOBAL_SPATIAL_FOUNDATION_CONTRACT_V1.md</x:v>
+      </x:c>
+      <x:c r="H136" t="str"/>
+      <x:c r="I136" t="str"/>
+      <x:c r="J136" t="str">
+        <x:v>Map|GIS|Cell|Region|Simulation|Terrain|Streaming|Storage|Persistence|Presentation</x:v>
+      </x:c>
+      <x:c r="K136" t="str">
+        <x:v>Keep Global Cell as the final world-space fact while allowing benchmark-driven technical partition sizes.</x:v>
+      </x:c>
+      <x:c r="L136" t="str"/>
+      <x:c r="M136" t="str"/>
+    </x:row>
+    <x:row r="137">
+      <x:c r="A137" t="str">
+        <x:v>decision.region-cell-boundary.05.v1</x:v>
+      </x:c>
+      <x:c r="B137" t="str">
+        <x:v>GlobalSpatialFoundation</x:v>
+      </x:c>
+      <x:c r="C137" t="str">
+        <x:v>Region and technical-block semantic decision 5</x:v>
+      </x:c>
+      <x:c r="D137" t="str">
+        <x:v>Region Polygon is derived or reference-only.</x:v>
+      </x:c>
+      <x:c r="E137" t="str">
+        <x:v>ACCEPTED</x:v>
+      </x:c>
+      <x:c r="F137" t="str">
+        <x:v>2026-08-15</x:v>
+      </x:c>
+      <x:c r="G137" t="str">
+        <x:v>Docs/HISTORICAL_WORLD_REFERENCE/WORLD_GLOBAL_ORIGIN_CELL_GRID_AND_SPATIAL_CONTINUITY_V1/GLOBAL_SPATIAL_FOUNDATION_CONTRACT_V1.md</x:v>
+      </x:c>
+      <x:c r="H137" t="str"/>
+      <x:c r="I137" t="str"/>
+      <x:c r="J137" t="str">
+        <x:v>Map|GIS|Cell|Region|Simulation|Terrain|Streaming|Storage|Persistence|Presentation</x:v>
+      </x:c>
+      <x:c r="K137" t="str">
+        <x:v>Keep Global Cell as the final world-space fact while allowing benchmark-driven technical partition sizes.</x:v>
+      </x:c>
+      <x:c r="L137" t="str"/>
+      <x:c r="M137" t="str"/>
+    </x:row>
+    <x:row r="138">
+      <x:c r="A138" t="str">
+        <x:v>decision.region-cell-boundary.06.v1</x:v>
+      </x:c>
+      <x:c r="B138" t="str">
+        <x:v>GlobalSpatialFoundation</x:v>
+      </x:c>
+      <x:c r="C138" t="str">
+        <x:v>Region and technical-block semantic decision 6</x:v>
+      </x:c>
+      <x:c r="D138" t="str">
+        <x:v>Technical Region is independent from AdministrativeRegion.</x:v>
+      </x:c>
+      <x:c r="E138" t="str">
+        <x:v>ACCEPTED</x:v>
+      </x:c>
+      <x:c r="F138" t="str">
+        <x:v>2026-08-15</x:v>
+      </x:c>
+      <x:c r="G138" t="str">
+        <x:v>Docs/HISTORICAL_WORLD_REFERENCE/WORLD_GLOBAL_ORIGIN_CELL_GRID_AND_SPATIAL_CONTINUITY_V1/GLOBAL_SPATIAL_FOUNDATION_CONTRACT_V1.md</x:v>
+      </x:c>
+      <x:c r="H138" t="str"/>
+      <x:c r="I138" t="str"/>
+      <x:c r="J138" t="str">
+        <x:v>Map|GIS|Cell|Region|Simulation|Terrain|Streaming|Storage|Persistence|Presentation</x:v>
+      </x:c>
+      <x:c r="K138" t="str">
+        <x:v>Keep Global Cell as the final world-space fact while allowing benchmark-driven technical partition sizes.</x:v>
+      </x:c>
+      <x:c r="L138" t="str"/>
+      <x:c r="M138" t="str"/>
+    </x:row>
+    <x:row r="139">
+      <x:c r="A139" t="str">
+        <x:v>decision.region-cell-boundary.07.v1</x:v>
+      </x:c>
+      <x:c r="B139" t="str">
+        <x:v>GlobalSpatialFoundation</x:v>
+      </x:c>
+      <x:c r="C139" t="str">
+        <x:v>Region and technical-block semantic decision 7</x:v>
+      </x:c>
+      <x:c r="D139" t="str">
+        <x:v>Chunk is a technical concept, not an authoritative world-space entity.</x:v>
+      </x:c>
+      <x:c r="E139" t="str">
+        <x:v>ACCEPTED</x:v>
+      </x:c>
+      <x:c r="F139" t="str">
+        <x:v>2026-08-15</x:v>
+      </x:c>
+      <x:c r="G139" t="str">
+        <x:v>Docs/HISTORICAL_WORLD_REFERENCE/WORLD_GLOBAL_ORIGIN_CELL_GRID_AND_SPATIAL_CONTINUITY_V1/GLOBAL_SPATIAL_FOUNDATION_CONTRACT_V1.md</x:v>
+      </x:c>
+      <x:c r="H139" t="str"/>
+      <x:c r="I139" t="str"/>
+      <x:c r="J139" t="str">
+        <x:v>Map|GIS|Cell|Region|Simulation|Terrain|Streaming|Storage|Persistence|Presentation</x:v>
+      </x:c>
+      <x:c r="K139" t="str">
+        <x:v>Keep Global Cell as the final world-space fact while allowing benchmark-driven technical partition sizes.</x:v>
+      </x:c>
+      <x:c r="L139" t="str"/>
+      <x:c r="M139" t="str"/>
+    </x:row>
+    <x:row r="140">
+      <x:c r="A140" t="str">
+        <x:v>decision.region-cell-boundary.08.v1</x:v>
+      </x:c>
+      <x:c r="B140" t="str">
+        <x:v>GlobalSpatialFoundation</x:v>
+      </x:c>
+      <x:c r="C140" t="str">
+        <x:v>Region and technical-block semantic decision 8</x:v>
+      </x:c>
+      <x:c r="D140" t="str">
+        <x:v>16x16 remains a spatial or simulation aggregation scale but is not automatically the Terrain or Streaming unit.</x:v>
+      </x:c>
+      <x:c r="E140" t="str">
+        <x:v>ACCEPTED</x:v>
+      </x:c>
+      <x:c r="F140" t="str">
+        <x:v>2026-08-15</x:v>
+      </x:c>
+      <x:c r="G140" t="str">
+        <x:v>Docs/HISTORICAL_WORLD_REFERENCE/WORLD_GLOBAL_ORIGIN_CELL_GRID_AND_SPATIAL_CONTINUITY_V1/GLOBAL_SPATIAL_FOUNDATION_CONTRACT_V1.md</x:v>
+      </x:c>
+      <x:c r="H140" t="str"/>
+      <x:c r="I140" t="str"/>
+      <x:c r="J140" t="str">
+        <x:v>Map|GIS|Cell|Region|Simulation|Terrain|Streaming|Storage|Persistence|Presentation</x:v>
+      </x:c>
+      <x:c r="K140" t="str">
+        <x:v>Keep Global Cell as the final world-space fact while allowing benchmark-driven technical partition sizes.</x:v>
+      </x:c>
+      <x:c r="L140" t="str"/>
+      <x:c r="M140" t="str"/>
+    </x:row>
+    <x:row r="141">
+      <x:c r="A141" t="str">
+        <x:v>decision.region-cell-boundary.09.v1</x:v>
+      </x:c>
+      <x:c r="B141" t="str">
+        <x:v>GlobalSpatialFoundation</x:v>
+      </x:c>
+      <x:c r="C141" t="str">
+        <x:v>Region and technical-block semantic decision 9</x:v>
+      </x:c>
+      <x:c r="D141" t="str">
+        <x:v>Terrain Tile, Streaming Unit, Simulation Aggregation Block and Storage Block may use different technical sizes.</x:v>
+      </x:c>
+      <x:c r="E141" t="str">
+        <x:v>ACCEPTED</x:v>
+      </x:c>
+      <x:c r="F141" t="str">
+        <x:v>2026-08-15</x:v>
+      </x:c>
+      <x:c r="G141" t="str">
+        <x:v>Docs/HISTORICAL_WORLD_REFERENCE/WORLD_GLOBAL_ORIGIN_CELL_GRID_AND_SPATIAL_CONTINUITY_V1/GLOBAL_SPATIAL_FOUNDATION_CONTRACT_V1.md</x:v>
+      </x:c>
+      <x:c r="H141" t="str"/>
+      <x:c r="I141" t="str"/>
+      <x:c r="J141" t="str">
+        <x:v>Map|GIS|Cell|Region|Simulation|Terrain|Streaming|Storage|Persistence|Presentation</x:v>
+      </x:c>
+      <x:c r="K141" t="str">
+        <x:v>Keep Global Cell as the final world-space fact while allowing benchmark-driven technical partition sizes.</x:v>
+      </x:c>
+      <x:c r="L141" t="str"/>
+      <x:c r="M141" t="str"/>
+    </x:row>
+    <x:row r="142">
+      <x:c r="A142" t="str">
+        <x:v>decision.region-cell-boundary.10.v1</x:v>
+      </x:c>
+      <x:c r="B142" t="str">
+        <x:v>GlobalSpatialFoundation</x:v>
+      </x:c>
+      <x:c r="C142" t="str">
+        <x:v>Region and technical-block semantic decision 10</x:v>
+      </x:c>
+      <x:c r="D142" t="str">
+        <x:v>No technical block may modify Stable Global Cell identity.</x:v>
+      </x:c>
+      <x:c r="E142" t="str">
+        <x:v>ACCEPTED</x:v>
+      </x:c>
+      <x:c r="F142" t="str">
+        <x:v>2026-08-15</x:v>
+      </x:c>
+      <x:c r="G142" t="str">
+        <x:v>Docs/HISTORICAL_WORLD_REFERENCE/WORLD_GLOBAL_ORIGIN_CELL_GRID_AND_SPATIAL_CONTINUITY_V1/GLOBAL_SPATIAL_FOUNDATION_CONTRACT_V1.md</x:v>
+      </x:c>
+      <x:c r="H142" t="str"/>
+      <x:c r="I142" t="str"/>
+      <x:c r="J142" t="str">
+        <x:v>Map|GIS|Cell|Region|Simulation|Terrain|Streaming|Storage|Persistence|Presentation</x:v>
+      </x:c>
+      <x:c r="K142" t="str">
+        <x:v>Keep Global Cell as the final world-space fact while allowing benchmark-driven technical partition sizes.</x:v>
+      </x:c>
+      <x:c r="L142" t="str"/>
+      <x:c r="M142" t="str"/>
+    </x:row>
+    <x:row r="143">
+      <x:c r="A143" t="str">
+        <x:v>DEC-MAP-STYLE-D-V2-001</x:v>
+      </x:c>
+      <x:c r="B143" t="str">
+        <x:v>MapPresentation</x:v>
+      </x:c>
+      <x:c r="C143" t="str">
+        <x:v>Global Cell resolution is not visual terrain resolution</x:v>
+      </x:c>
+      <x:c r="D143" t="str">
+        <x:v>Style D may refine presentation vertices at REGION/CITY/CLOSE levels without creating simulation SubCells or changing 2000m Cell facts.</x:v>
+      </x:c>
+      <x:c r="E143" t="str">
+        <x:v>FROZEN</x:v>
+      </x:c>
+      <x:c r="F143" t="str">
+        <x:v>2026-08-16</x:v>
+      </x:c>
+      <x:c r="G143" t="str">
+        <x:v>Docs/HISTORICAL_WORLD_REFERENCE/HAN_WORLD_STYLE_D_STRATEGIC_LANDSCAPE_VISUAL_REFINEMENT_V2/STYLE_D_STRATEGIC_LANDSCAPE_VISUAL_REFINEMENT_V2_REPORT.md</x:v>
+      </x:c>
+      <x:c r="H143"/>
+      <x:c r="I143" t="str">
+        <x:v>GLOBAL_SPATIAL_FOUNDATION_CONTRACT_V1.md|MAP_ART_RESOURCE_PLAN.md|GAME_SYSTEMS_MASTER_AND_STATUS.md</x:v>
+      </x:c>
+      <x:c r="J143" t="str">
+        <x:v>Map|Presentation|SpatialFoundation</x:v>
+      </x:c>
+      <x:c r="K143" t="str">
+        <x:v>User task and V2 implementation contract</x:v>
+      </x:c>
+      <x:c r="L143" t="str">
+        <x:v>User visual review pending</x:v>
+      </x:c>
+      <x:c r="M143" t="str">
+        <x:v>No nationwide rollout in this task</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:L1"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R763e48be991a4873"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R41c91510527845e4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>